<commit_message>
Resolver-Pass 5 setup: fill driver config + Call-3 author backfill
- resolver-pass.config.json: replace NNN/REPLACE placeholders for Pass 5 (089), add facet-catalog.json to phase-4 scope + Call-2/3 trigger clause (incl. facet_values DB-seed dependency note)
- book-roster.json + Warhammer_Books_SSOT.xlsx: backfill authors W40K-0206 (Steven B. Fischer), W40K-0244 (Mike Vincent) via import:ssot-roster
- sessions/README.md: active-threads update for Brief 089
- add Brief 089 arch brief
</commit_message>
<xml_diff>
--- a/scripts/seed-data/source/Warhammer_Books_SSOT.xlsx
+++ b/scripts/seed-data/source/Warhammer_Books_SSOT.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="1" r:id="Rfd2bfd18733d40f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Links" sheetId="2" r:id="R9c8fbfa1a98f417d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Comparison" sheetId="3" r:id="R4f0bba3a4c03492d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unmapped Collections" sheetId="4" r:id="R5d8518f7a83a4206"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R9a654b57de324c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="R1a56048cfc784aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Books" sheetId="1" r:id="R35829f91ee7142aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Collection Links" sheetId="2" r:id="Rf7adef8a144241b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Comparison" sheetId="3" r:id="R93fbd20898c848ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unmapped Collections" sheetId="4" r:id="R9f0dc7e939794083"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R106b3a14f7f64f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="6" r:id="Rf9c077bad7744baa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,13 +26,13 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="10"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -49,7 +49,7 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="1F2937"/>
+        <x:fgColor rgb="FF1F2937"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1002,7 +1002,7 @@
         <x:v>Warhammer 40k</x:v>
       </x:c>
       <x:c r="D16" s="7" t="str">
-        <x:v>Death of Glory</x:v>
+        <x:v>Death or Glory</x:v>
       </x:c>
       <x:c r="E16" s="7" t="str">
         <x:v>Sandy Mitchell</x:v>
@@ -8898,7 +8898,9 @@
       <x:c r="D207" s="7" t="str">
         <x:v>Broken Crusade</x:v>
       </x:c>
-      <x:c r="E207" s="7" t="str"/>
+      <x:c r="E207" s="7" t="str">
+        <x:v>Steven B. Fischer</x:v>
+      </x:c>
       <x:c r="F207" s="7" t="str">
         <x:v>2024</x:v>
       </x:c>
@@ -10510,7 +10512,9 @@
       <x:c r="D245" s="7" t="str">
         <x:v>The Remnant Blade</x:v>
       </x:c>
-      <x:c r="E245" s="7" t="str"/>
+      <x:c r="E245" s="7" t="str">
+        <x:v>Mike Vincent</x:v>
+      </x:c>
       <x:c r="F245" s="7" t="str">
         <x:v>2025</x:v>
       </x:c>
@@ -35784,7 +35788,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R875b823741bb46d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7a642a9c3244d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -41952,7 +41956,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ea89ed6aec644d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71a7c9c7df7746fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -42079,7 +42083,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b40ddcc11454a7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a0f903ae66b44b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43525,7 +43529,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R074f66da3b044f4a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9534c68bed47419f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43619,7 +43623,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9463318ac604456e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8780d5035e9d42d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -43683,7 +43687,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8915534db9449d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ae0c6591eb343f9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>